<commit_message>
Werkboek bijgewerkt naar de kopie van 07-09
Het werkboek op de site was dat van 31 augustus. Deze kopie verschilt daarvan
op drie plekken: de vraag bij de keten-analyse is korter geformuleerd, kolom B
op Instellingen is breder, en de databalk op het Dashboard is rood in plaats
van grijs.

De bron verandert niet mee: haal_bron.py haalt uit dit bestand exact dezelfde
eisteksten, maatregelen, niveaus en keuzelijsten, dus van csir.json wijzigt
alleen werkboek_sha256. De downloadpagina toont die vingerafdruk, dus die loopt
vanzelf mee.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VkfRod3NBVwKtMkwioRN7Z
</commit_message>
<xml_diff>
--- a/werkboek/csir-control-register.xlsx
+++ b/werkboek/csir-control-register.xlsx
@@ -1579,7 +1579,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="4" customWidth="1" min="5" max="5"/>
@@ -1668,7 +1668,7 @@
     <row r="12">
       <c r="B12" s="58" t="inlineStr">
         <is>
-          <t>Bedient/beheert dit object andere objecten?</t>
+          <t>Bedient of beheert andere objecten?</t>
         </is>
       </c>
       <c r="C12" s="88" t="n"/>
@@ -2952,11 +2952,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J7:J10">
-    <cfRule type="dataBar" priority="6">
+    <cfRule type="dataBar" priority="4">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="1"/>
-        <color rgb="FF7A8B93"/>
+        <color rgb="FFD90727"/>
       </dataBar>
     </cfRule>
   </conditionalFormatting>

</xml_diff>